<commit_message>
Licitaciones: corrida 2026-09-20 19:30 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -850,7 +850,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1443,13 +1443,19 @@
       <c r="N9" s="3" t="n">
         <v>5000000000</v>
       </c>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="4" t="n"/>
-      <c r="Q9" s="5" t="n"/>
+      <c r="O9" s="3" t="n">
+        <v>16881478745</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>3.376295749</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>27</v>
+      </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>TASA DE CORTE: %</t>
+          <t>TASA DE CORTE: 27.00%</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1530,7 +1536,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1571,13 +1577,19 @@
       <c r="N10" s="3" t="n">
         <v>5000000000</v>
       </c>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="4" t="n"/>
-      <c r="Q10" s="5" t="n"/>
+      <c r="O10" s="3" t="n">
+        <v>257644579</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0.0515289158</v>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>5.5</v>
+      </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 5.50%</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1658,7 +1670,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Cancelada/Suspendida</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1786,7 +1798,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1827,13 +1839,17 @@
       <c r="N12" s="3" t="n">
         <v>5000000000</v>
       </c>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="4" t="n"/>
+      <c r="O12" s="3" t="n">
+        <v>50031830843</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>10.0063661686</v>
+      </c>
       <c r="Q12" s="5" t="n"/>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE: $</t>
+          <t>PRECIO DE CORTE: 1.043388</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1914,7 +1930,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1955,13 +1971,17 @@
       <c r="N13" s="3" t="n">
         <v>5000000000</v>
       </c>
-      <c r="O13" s="3" t="n"/>
-      <c r="P13" s="4" t="n"/>
+      <c r="O13" s="3" t="n">
+        <v>7794965725</v>
+      </c>
+      <c r="P13" s="4" t="n">
+        <v>1.558993145</v>
+      </c>
       <c r="Q13" s="5" t="n"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE: $</t>
+          <t>PRECIO DE CORTE: 1.029210</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -2042,7 +2062,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2083,13 +2103,19 @@
       <c r="N14" s="3" t="n">
         <v>100000000</v>
       </c>
-      <c r="O14" s="3" t="n"/>
-      <c r="P14" s="4" t="n"/>
-      <c r="Q14" s="5" t="n"/>
+      <c r="O14" s="3" t="n">
+        <v>233654373</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>2.33654373</v>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>6.25</v>
+      </c>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>TASA DE CORTE: 6.25%</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -2170,7 +2196,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2211,13 +2237,17 @@
       <c r="N15" s="3" t="n">
         <v>18600000000</v>
       </c>
-      <c r="O15" s="3" t="n"/>
-      <c r="P15" s="4" t="n"/>
+      <c r="O15" s="3" t="n">
+        <v>18600000000</v>
+      </c>
+      <c r="P15" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q15" s="5" t="n"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE VDFA: % / PRECIO DE CORTE VDFB: %</t>
+          <t>PRECIO DE CORTE VDFA: $ 1.0050 POR CADA V/N $ 1 / PRECIO DE CORTE VDFB: $ 1.00 POR CADA V/N $ 1</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2293,7 +2323,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2334,13 +2364,19 @@
       <c r="N16" s="3" t="n">
         <v>9883265871</v>
       </c>
-      <c r="O16" s="3" t="n"/>
-      <c r="P16" s="4" t="n"/>
-      <c r="Q16" s="5" t="n"/>
+      <c r="O16" s="3" t="n">
+        <v>9883265871</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="5" t="n">
+        <v>26.67</v>
+      </c>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
-          <t>VDFA: TIR DE CORTE % / VDFB: TIR DE CORTE % / CP PRECIO DE CORTE: %</t>
+          <t>VDFA: TIR DE CORTE 26.67% / VDFB: TIR DE CORTE 29.77% / CP PRECIO DE CORTE: 100%</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -11877,7 +11913,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Finalizada</t>
+          <t>Cancelada/Suspendida</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-09-22 21:56 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,17 @@
       <c r="N2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>2418615422</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>2418615422</v>
+      </c>
       <c r="Q2" s="5" t="n"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>PRECIO DE CORTE: $ 993.58</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -864,13 +868,17 @@
       <c r="N3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="4" t="n"/>
+      <c r="O3" s="3" t="n">
+        <v>843337067</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>843337067</v>
+      </c>
       <c r="Q3" s="5" t="n"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>PRECIO DE CORTE: $ 989.98</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -987,13 +995,17 @@
       <c r="N4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="4" t="n"/>
+      <c r="O4" s="3" t="n">
+        <v>70179576</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>70179576</v>
+      </c>
       <c r="Q4" s="5" t="n"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>PRECIO DE CORTE: $ 846.60</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1441,8 +1453,12 @@
       <c r="N8" s="3" t="n">
         <v>4000000000</v>
       </c>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="4" t="n"/>
+      <c r="O8" s="3" t="n">
+        <v>2071428571</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0.5178571427500001</v>
+      </c>
       <c r="Q8" s="5" t="n"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
@@ -1569,8 +1585,12 @@
       <c r="N9" s="3" t="n">
         <v>2000000000</v>
       </c>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="4" t="n"/>
+      <c r="O9" s="3" t="n">
+        <v>2071428571</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>1.0357142855</v>
+      </c>
       <c r="Q9" s="5" t="n"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
@@ -1697,8 +1717,12 @@
       <c r="N10" s="3" t="n">
         <v>2000000000</v>
       </c>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="4" t="n"/>
+      <c r="O10" s="3" t="n">
+        <v>2071428571</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>1.0357142855</v>
+      </c>
       <c r="Q10" s="5" t="n"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
@@ -1953,13 +1977,19 @@
       <c r="N12" s="3" t="n">
         <v>30000000000</v>
       </c>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="4" t="n"/>
-      <c r="Q12" s="5" t="n"/>
+      <c r="O12" s="3" t="n">
+        <v>69895900000</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>2.329863333333333</v>
+      </c>
+      <c r="Q12" s="5" t="n">
+        <v>7</v>
+      </c>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>MARGEN APLICABLE: %</t>
+          <t>MARGEN APLICABLE: 7.00 %</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -2081,13 +2111,19 @@
       <c r="N13" s="3" t="n">
         <v>1000000000</v>
       </c>
-      <c r="O13" s="3" t="n"/>
-      <c r="P13" s="4" t="n"/>
-      <c r="Q13" s="5" t="n"/>
+      <c r="O13" s="3" t="n">
+        <v>2071428571</v>
+      </c>
+      <c r="P13" s="4" t="n">
+        <v>2.071428571</v>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>-0.5</v>
+      </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: -0.5%</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-09-23 22:10 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,19 @@
       <c r="N2" s="3" t="n">
         <v>40000000</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="5" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>35903000</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>0.897575</v>
+      </c>
+      <c r="Q2" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>TASA DE CORTE: %</t>
+          <t>TASA DE CORTE: 6.00%</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -869,13 +875,19 @@
       <c r="N3" s="3" t="n">
         <v>4000000000</v>
       </c>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="4" t="n"/>
-      <c r="Q3" s="5" t="n"/>
+      <c r="O3" s="3" t="n">
+        <v>9357142856</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>2.339285714</v>
+      </c>
+      <c r="Q3" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 0.00 %</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -997,13 +1009,19 @@
       <c r="N4" s="3" t="n">
         <v>5000000000</v>
       </c>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="4" t="n"/>
-      <c r="Q4" s="5" t="n"/>
+      <c r="O4" s="3" t="n">
+        <v>8000000000</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>7.5</v>
+      </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 7.50% N.A.</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1125,13 +1143,19 @@
       <c r="N5" s="3" t="n">
         <v>10000000000</v>
       </c>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="4" t="n"/>
-      <c r="Q5" s="5" t="n"/>
+      <c r="O5" s="3" t="n">
+        <v>30009162500</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>3.00091625</v>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>4.5</v>
+      </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 4.50%</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1181,7 +1205,7 @@
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>Las Obligaciones Negociables serán suscriptas e integradas en Pesos.</t>
+          <t>Las Obligaciones Negociables Serie 69 serán Suscriptas, Integradas y Pagaderas en Pesos.</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr"/>
@@ -1257,11 +1281,7 @@
       <c r="P6" s="4" t="n"/>
       <c r="Q6" s="5" t="n"/>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>TEM DE CORTE: %</t>
-        </is>
-      </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
           <t>TEM</t>
@@ -1309,7 +1329,7 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>Las ON serán suscriptas e integradas en Pesos.</t>
+          <t>Las Obligaciones Negociables Serie 70 serán Suscriptas, Integradas y Pagaderas en Pesos.</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr"/>

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-09-24 22:11 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,19 @@
       <c r="N2" s="3" t="n">
         <v>10000000</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="5" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>30881342</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>3.0881342</v>
+      </c>
+      <c r="Q2" s="5" t="n">
+        <v>6.5</v>
+      </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>TASA DE CORTE: %</t>
+          <t>TASA DE CORTE: 6.50 %</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -865,13 +871,19 @@
       <c r="N3" s="3" t="n">
         <v>20000000</v>
       </c>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="4" t="n"/>
-      <c r="Q3" s="5" t="n"/>
+      <c r="O3" s="3" t="n">
+        <v>20065298</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>1.0032649</v>
+      </c>
+      <c r="Q3" s="5" t="n">
+        <v>5.25</v>
+      </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>TASA DE CORTE: %</t>
+          <t>TASA DE CORTE: 5.25%</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -993,13 +1005,19 @@
       <c r="N4" s="3" t="n">
         <v>3000000</v>
       </c>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="4" t="n"/>
-      <c r="Q4" s="5" t="n"/>
+      <c r="O4" s="3" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>100</v>
+      </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>ADHESIÓN 100%</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1117,13 +1135,17 @@
       <c r="N5" s="3" t="n">
         <v>20000000</v>
       </c>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="4" t="n"/>
+      <c r="O5" s="3" t="n">
+        <v>20724373</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>1.03621865</v>
+      </c>
       <c r="Q5" s="5" t="n"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>PRECIO DE CORTE: $ 1.0077</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1245,8 +1267,12 @@
       <c r="N6" s="3" t="n">
         <v>75000000</v>
       </c>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="4" t="n"/>
+      <c r="O6" s="3" t="n">
+        <v>20724373</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0.2763249733333333</v>
+      </c>
       <c r="Q6" s="5" t="n"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-09-29 22:54 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,19 @@
       <c r="N2" s="3" t="n">
         <v>8877516</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="5" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>8877516</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="5" t="n">
+        <v>100</v>
+      </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>100 %</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-01 23:04 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -1116,13 +1116,19 @@
       <c r="N7" s="3" t="n">
         <v>40000000</v>
       </c>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="4" t="n"/>
-      <c r="Q7" s="5" t="n"/>
+      <c r="O7" s="3" t="n">
+        <v>43370436</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>1.0842609</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>5.69</v>
+      </c>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>TASA DE CORTE: 5.69%</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1244,13 +1250,19 @@
       <c r="N8" s="3" t="n">
         <v>40000000</v>
       </c>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="4" t="n"/>
-      <c r="Q8" s="5" t="n"/>
+      <c r="O8" s="3" t="n">
+        <v>55408498875</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>1385.212471875</v>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>4.95</v>
+      </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>MARGEN DE CORTE: 4.95%</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1372,13 +1384,19 @@
       <c r="N9" s="3" t="n">
         <v>13270000000</v>
       </c>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="4" t="n"/>
-      <c r="Q9" s="5" t="n"/>
+      <c r="O9" s="3" t="n">
+        <v>13270000000</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>28.19</v>
+      </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>TIR DE CORTE: VDFA 28.19% / VDFB 33.41% / VDFC 40.74 %</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-02 18:19 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -1547,7 +1547,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -12740,7 +12740,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Finalizada</t>
+          <t>Cancelada/Suspendida</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-05 21:13 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-06 22:57 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,19 @@
       <c r="N2" s="3" t="n">
         <v>200000000000</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="5" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>200000000000</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="5" t="n">
+        <v>2.71</v>
+      </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>TRAMO 1: SPREAD P.P. 2.71% - TRAMO 2: SPREAD P.P. 4.79%</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -864,13 +870,19 @@
       <c r="N3" s="3" t="n">
         <v>30000000</v>
       </c>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="4" t="n"/>
-      <c r="Q3" s="5" t="n"/>
+      <c r="O3" s="3" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>1.666666666666667</v>
+      </c>
+      <c r="Q3" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>TASA DE CORTE: 6.00%</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -992,13 +1004,19 @@
       <c r="N4" s="3" t="n">
         <v>2500000000</v>
       </c>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="4" t="n"/>
-      <c r="Q4" s="5" t="n"/>
+      <c r="O4" s="3" t="n">
+        <v>3500000000</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 0.00%</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1120,13 +1138,19 @@
       <c r="N5" s="3" t="n">
         <v>10000000000</v>
       </c>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="4" t="n"/>
-      <c r="Q5" s="5" t="n"/>
+      <c r="O5" s="3" t="n">
+        <v>40530000000</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>4.053</v>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>4.65</v>
+      </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 4.65%</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-08 00:53 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,19 @@
       <c r="N2" s="3" t="n">
         <v>10000000000</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="5" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>20000000000</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="5" t="n">
+        <v>4.49</v>
+      </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 4.49%</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-09 23:08 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,19 @@
       <c r="N2" s="3" t="n">
         <v>3614615169</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="5" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>3614615169</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="5" t="n">
+        <v>101.68</v>
+      </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE: VDFA % / VDFB % / VDFC % / CP %</t>
+          <t>PRECIO DE CORTE: VDFA 101.68% / VDFB 100% / VDFC 100% / CP 150%</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-12 21:41 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -700,7 +700,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-14 22:11 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,17 @@
       <c r="N2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>726905677</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>726905677</v>
+      </c>
       <c r="Q2" s="5" t="n"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE: %</t>
+          <t>PRECIO DE CORTE: $ 946.46</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -869,13 +873,17 @@
       <c r="N3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="4" t="n"/>
+      <c r="O3" s="3" t="n">
+        <v>1055629289724</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>1055629289724</v>
+      </c>
       <c r="Q3" s="5" t="n"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE: %</t>
+          <t>PRECIO DE CORTE POR CADA VNO $ 1.000: $ 1096.00</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -997,13 +1005,17 @@
       <c r="N4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="4" t="n"/>
+      <c r="O4" s="3" t="n">
+        <v>1941291135533</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>1941291135533</v>
+      </c>
       <c r="Q4" s="5" t="n"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE: %</t>
+          <t>PRECIO DE CORTE POR CADA VNO $ 1.000: $ 878.00</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1125,13 +1137,17 @@
       <c r="N5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="4" t="n"/>
+      <c r="O5" s="3" t="n">
+        <v>2597092832639</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>2597092832639</v>
+      </c>
       <c r="Q5" s="5" t="n"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE: %</t>
+          <t>PRECIO DE CORTE POR CADA VNO $ 1.000: $ 1041.92</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1253,13 +1269,19 @@
       <c r="N6" s="3" t="n">
         <v>1000000000</v>
       </c>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="4" t="n"/>
-      <c r="Q6" s="5" t="n"/>
+      <c r="O6" s="3" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="5" t="n">
+        <v>-0.03</v>
+      </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: -0,03%</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1381,13 +1403,19 @@
       <c r="N7" s="3" t="n">
         <v>14593147882</v>
       </c>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="4" t="n"/>
-      <c r="Q7" s="5" t="n"/>
+      <c r="O7" s="3" t="n">
+        <v>14593147882</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>4.25</v>
+      </c>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE VDFA: % / VDFB: % / VDFC: %</t>
+          <t>MARGEN DE CORTE VDFA: 4.25 % / VDFB: 12.0 % / VDFC: 8.00 %</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-15 22:05 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -816,13 +816,17 @@
       <c r="N3" s="3" t="n">
         <v>5000000000</v>
       </c>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="4" t="n"/>
+      <c r="O3" s="3" t="n">
+        <v>48828558222</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>9.7657116444</v>
+      </c>
       <c r="Q3" s="5" t="n"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE: $</t>
+          <t>PRECIO DE CORTE: 1.050110</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -944,13 +948,17 @@
       <c r="N4" s="3" t="n">
         <v>5000000000</v>
       </c>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="4" t="n"/>
+      <c r="O4" s="3" t="n">
+        <v>10319980416</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>2.0639960832</v>
+      </c>
       <c r="Q4" s="5" t="n"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE: $</t>
+          <t>PRECIO DE CORTE: 1.021017</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1072,13 +1080,19 @@
       <c r="N5" s="3" t="n">
         <v>5000000000</v>
       </c>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="4" t="n"/>
-      <c r="Q5" s="5" t="n"/>
+      <c r="O5" s="3" t="n">
+        <v>2215298746</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0.4430597492</v>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>27</v>
+      </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>TASA DE CORTE: %</t>
+          <t>TASA DE CORTE: 27.00%</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1200,13 +1214,19 @@
       <c r="N6" s="3" t="n">
         <v>5000000000</v>
       </c>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="4" t="n"/>
-      <c r="Q6" s="5" t="n"/>
+      <c r="O6" s="3" t="n">
+        <v>1372468535</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0.274493707</v>
+      </c>
+      <c r="Q6" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 6.00%</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1331,10 +1351,14 @@
       <c r="O7" s="3" t="n"/>
       <c r="P7" s="4" t="n"/>
       <c r="Q7" s="5" t="n"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>DESIERTA</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1584,13 +1608,19 @@
       <c r="N9" s="3" t="n">
         <v>2000000000</v>
       </c>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="4" t="n"/>
-      <c r="Q9" s="5" t="n"/>
+      <c r="O9" s="3" t="n">
+        <v>3087272725</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>1.5436363625</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 1%</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-20 22:12 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,17 @@
       <c r="N2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>1043079706</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>1043079706</v>
+      </c>
       <c r="Q2" s="5" t="n"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>PRECIO DE CORTE: $ 990.00</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -869,13 +873,17 @@
       <c r="N3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="4" t="n"/>
+      <c r="O3" s="3" t="n">
+        <v>2680518062</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>2680518062</v>
+      </c>
       <c r="Q3" s="5" t="n"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>PRECIO DE CORTE: $ 992.07</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -997,13 +1005,17 @@
       <c r="N4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="4" t="n"/>
+      <c r="O4" s="3" t="n">
+        <v>206121216</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>206121216</v>
+      </c>
       <c r="Q4" s="5" t="n"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>PRECIO DE CORTE: $ 972.00</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1125,13 +1137,19 @@
       <c r="N5" s="3" t="n">
         <v>50000000000</v>
       </c>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="4" t="n"/>
-      <c r="Q5" s="5" t="n"/>
+      <c r="O5" s="3" t="n">
+        <v>211505165000</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>4.2301033</v>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>9.75</v>
+      </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 9.75%</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1253,13 +1271,17 @@
       <c r="N6" s="3" t="n">
         <v>2000000000</v>
       </c>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="4" t="n"/>
+      <c r="O6" s="3" t="n">
+        <v>431776717935</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>215.8883589675</v>
+      </c>
       <c r="Q6" s="5" t="n"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE:</t>
+          <t>PRECIO DE CORTE: 0.981552</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1381,13 +1403,17 @@
       <c r="N7" s="3" t="n">
         <v>2000000000</v>
       </c>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="4" t="n"/>
+      <c r="O7" s="3" t="n">
+        <v>143300642222</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>71.650321111</v>
+      </c>
       <c r="Q7" s="5" t="n"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE:</t>
+          <t>PRECIO DE CORTE: 0.96235</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1509,13 +1535,19 @@
       <c r="N8" s="3" t="n">
         <v>2000000000</v>
       </c>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="4" t="n"/>
-      <c r="Q8" s="5" t="n"/>
+      <c r="O8" s="3" t="n">
+        <v>1778858000</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0.889429</v>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>2.15</v>
+      </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
-          <t>TEM DE CORTE: %</t>
+          <t>TEM DE CORTE: 2.15%</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1637,13 +1669,19 @@
       <c r="N9" s="3" t="n">
         <v>2000000000</v>
       </c>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="4" t="n"/>
-      <c r="Q9" s="5" t="n"/>
+      <c r="O9" s="3" t="n">
+        <v>7426955780</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>3.71347789</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>4.75</v>
+      </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>TASA DE CORTE: %</t>
+          <t>TASA DE CORTE: 4.75%</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1765,13 +1803,19 @@
       <c r="N10" s="3" t="n">
         <v>2000000000</v>
       </c>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="4" t="n"/>
-      <c r="Q10" s="5" t="n"/>
+      <c r="O10" s="3" t="n">
+        <v>53278268612</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>26.639134306</v>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>4.75</v>
+      </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 4.75%</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1893,13 +1937,19 @@
       <c r="N11" s="3" t="n">
         <v>20000000000</v>
       </c>
-      <c r="O11" s="3" t="n"/>
-      <c r="P11" s="4" t="n"/>
-      <c r="Q11" s="5" t="n"/>
+      <c r="O11" s="3" t="n">
+        <v>29708890000</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>1.4854445</v>
+      </c>
+      <c r="Q11" s="5" t="n">
+        <v>3.99</v>
+      </c>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 3.99 %</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -2021,13 +2071,19 @@
       <c r="N12" s="3" t="n">
         <v>1000000</v>
       </c>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="4" t="n"/>
-      <c r="Q12" s="5" t="n"/>
+      <c r="O12" s="3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="5" t="n">
+        <v>9.25</v>
+      </c>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>TASA DE CORTE: %</t>
+          <t>TASA DE CORTE: 9.25%</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-22 17:55 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -978,7 +978,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-27 22:56 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,19 @@
       <c r="N2" s="3" t="n">
         <v>3000000000</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="5" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>3000000000</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="5" t="n">
+        <v>3.95</v>
+      </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 3.95%</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -869,13 +875,19 @@
       <c r="N3" s="3" t="n">
         <v>50000000</v>
       </c>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="4" t="n"/>
-      <c r="Q3" s="5" t="n"/>
+      <c r="O3" s="3" t="n">
+        <v>135917743471</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>2718.35486942</v>
+      </c>
+      <c r="Q3" s="5" t="n">
+        <v>5.5</v>
+      </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>MARGEN DE CORTE: 5.5%</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -993,13 +1005,19 @@
       <c r="N4" s="3" t="n">
         <v>50000000</v>
       </c>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="4" t="n"/>
-      <c r="Q4" s="5" t="n"/>
+      <c r="O4" s="3" t="n">
+        <v>68760964</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>1.37521928</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>5.75</v>
+      </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>TASA DE CORTE: 5.75%</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1117,13 +1135,17 @@
       <c r="N5" s="3" t="n">
         <v>21889463244</v>
       </c>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="4" t="n"/>
+      <c r="O5" s="3" t="n">
+        <v>21889463244</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q5" s="5" t="n"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>VDFA: PRECIO DE CORTE % / VDFB: PRECIO DE CORTE %</t>
+          <t>VDFA: PRECIO DE CORTE $ 0.9870 / VDFB: PRECIO DE CORTE $ 0.985924</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1240,13 +1262,19 @@
       <c r="N6" s="3" t="n">
         <v>2000000000</v>
       </c>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="4" t="n"/>
-      <c r="Q6" s="5" t="n"/>
+      <c r="O6" s="3" t="n">
+        <v>5000000000</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q6" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 0.00%</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-28 23:04 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,17 @@
       <c r="N2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>1203102518400</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>1203102518400</v>
+      </c>
       <c r="Q2" s="5" t="n"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE POR CADA VNO $ 1.000: $</t>
+          <t>PRECIO DE CORTE POR CADA VNO $ 1.000: $ 1.215</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -869,13 +873,17 @@
       <c r="N3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="4" t="n"/>
+      <c r="O3" s="3" t="n">
+        <v>3665004206129</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>3665004206129</v>
+      </c>
       <c r="Q3" s="5" t="n"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE POR CADA VNO $ 1.000: $</t>
+          <t>PRECIO DE CORTE POR CADA VNO $ 1.000: $ 964.5</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -997,13 +1005,17 @@
       <c r="N4" s="3" t="n">
         <v>6000000</v>
       </c>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="4" t="n"/>
+      <c r="O4" s="3" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q4" s="5" t="n"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE VDF:</t>
+          <t>PRECIO DE CORTE VDF: 0.9969</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1120,13 +1132,19 @@
       <c r="N5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="4" t="n"/>
-      <c r="Q5" s="5" t="n"/>
+      <c r="O5" s="3" t="n">
+        <v>2078223635336</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>2078223635336</v>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>2.1</v>
+      </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>TEM DE CORTE: %</t>
+          <t>TEM DE CORTE: 2.10%</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1248,13 +1266,17 @@
       <c r="N6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="4" t="n"/>
+      <c r="O6" s="3" t="n">
+        <v>481372844519</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>481372844519</v>
+      </c>
       <c r="Q6" s="5" t="n"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE POR CADA VNO $ 1.000:</t>
+          <t>PRECIO DE CORTE POR CADA VNO $ 1.000: $ 2.337</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1376,13 +1398,17 @@
       <c r="N7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="4" t="n"/>
+      <c r="O7" s="3" t="n">
+        <v>816939994213</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>816939994213</v>
+      </c>
       <c r="Q7" s="5" t="n"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE POR CADA VNO $ 1.000:</t>
+          <t>PRECIO DE CORTE POR CADA VNO $ 1.000: $ 1.017</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1504,13 +1530,17 @@
       <c r="N8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="4" t="n"/>
+      <c r="O8" s="3" t="n">
+        <v>1666204256</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>1666204256</v>
+      </c>
       <c r="Q8" s="5" t="n"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
-          <t>PRECIO DE CORTE POR CADA VNO USD 1.000: USD</t>
+          <t>PRECIO DE CORTE POR CADA VNO USD 1.000: USD 986</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1632,13 +1662,19 @@
       <c r="N9" s="3" t="n">
         <v>5000000</v>
       </c>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="4" t="n"/>
-      <c r="Q9" s="5" t="n"/>
+      <c r="O9" s="3" t="n">
+        <v>6108085</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>1.221617</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>6.5</v>
+      </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>TASA DE CORTE: %</t>
+          <t>TASA DE CORTE: 6.50%</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1760,13 +1796,19 @@
       <c r="N10" s="3" t="n">
         <v>5000000</v>
       </c>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="4" t="n"/>
-      <c r="Q10" s="5" t="n"/>
+      <c r="O10" s="3" t="n">
+        <v>17583000000</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>3516.6</v>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>MARGEN DE CORTE: %</t>
+          <t>MARGEN DE CORTE: 6.00%</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1883,13 +1925,19 @@
       <c r="N11" s="3" t="n">
         <v>200000000</v>
       </c>
-      <c r="O11" s="3" t="n"/>
-      <c r="P11" s="4" t="n"/>
-      <c r="Q11" s="5" t="n"/>
+      <c r="O11" s="3" t="n">
+        <v>220215000</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>1.101075</v>
+      </c>
+      <c r="Q11" s="5" t="n">
+        <v>6.5</v>
+      </c>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
-          <t>TASA DE CORTE: %</t>
+          <t>TASA DE CORTE: 6.5 %</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">

</xml_diff>

<commit_message>
Licitaciones: corrida 2026-10-29 23:12 UTC
</commit_message>
<xml_diff>
--- a/datos/licitaciones.xlsx
+++ b/datos/licitaciones.xlsx
@@ -741,13 +741,19 @@
       <c r="N2" s="3" t="n">
         <v>30000000</v>
       </c>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="5" t="n"/>
+      <c r="O2" s="3" t="n">
+        <v>56817670</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>1.893922333333333</v>
+      </c>
+      <c r="Q2" s="5" t="n">
+        <v>6.75</v>
+      </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>TASA DE CORTE: %</t>
+          <t>TASA DE CORTE: 6.75%</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">

</xml_diff>